<commit_message>
Fixed non-food demand for animal prods + errors in animal prod/by-prod calc, cream balance and demand parameter sheet (see also previous commit). Dairy parameters+calc still need checking
</commit_message>
<xml_diff>
--- a/data/prod_parameters/DemandAndConversions.xlsx
+++ b/data/prod_parameters/DemandAndConversions.xlsx
@@ -4877,7 +4877,7 @@
       </c>
       <c r="K183" s="13">
         <f>100-K184</f>
-        <v>93.25</v>
+        <v>97</v>
       </c>
       <c r="L183" s="11" t="s">
         <v>39</v>
@@ -4911,8 +4911,8 @@
         <v>89</v>
       </c>
       <c r="K184" s="13">
-        <f>(0.042-0.015)/0.4*100</f>
-        <v>6.75</v>
+        <f>(0.042-0.03)/0.4*100</f>
+        <v>3.0000000000000009</v>
       </c>
       <c r="L184" s="11" t="s">
         <v>39</v>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="K185" s="13">
         <f>(100-K186)*0.1</f>
-        <v>9.3250000000000011</v>
+        <v>9.7000000000000011</v>
       </c>
       <c r="L185" s="11" t="s">
         <v>39</v>
@@ -4976,8 +4976,8 @@
         <v>89</v>
       </c>
       <c r="K186" s="13">
-        <f>(0.042-0.015)/0.4*100</f>
-        <v>6.75</v>
+        <f>(0.042-0.03)/0.4*100</f>
+        <v>3.0000000000000009</v>
       </c>
       <c r="L186" s="11" t="s">
         <v>39</v>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="K187" s="13">
         <f>(100-K186)*0.9</f>
-        <v>83.924999999999997</v>
+        <v>87.3</v>
       </c>
       <c r="L187" s="11" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
Updated notebook and baseline scenario
</commit_message>
<xml_diff>
--- a/data/prod_parameters/DemandAndConversions.xlsx
+++ b/data/prod_parameters/DemandAndConversions.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="9870"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="9870" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1428" uniqueCount="303">
   <si>
     <t>parameter</t>
   </si>
@@ -8352,7 +8352,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -8485,29 +8485,12 @@
       <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>275</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adjusted starch potatoe non-food and exports
</commit_message>
<xml_diff>
--- a/data/prod_parameters/DemandAndConversions.xlsx
+++ b/data/prod_parameters/DemandAndConversions.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="335">
   <si>
     <t>parameter</t>
   </si>
@@ -1067,6 +1067,9 @@
   </si>
   <si>
     <t>Majs</t>
+  </si>
+  <si>
+    <t>Use total exports as import accounted for in food demand. OK?</t>
   </si>
 </sst>
 </file>
@@ -3219,13 +3222,13 @@
         <v>318</v>
       </c>
       <c r="K97" s="22">
-        <v>22400.2</v>
+        <v>32965.800000000003</v>
       </c>
       <c r="L97" t="s">
         <v>204</v>
       </c>
       <c r="M97" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="N97" t="s">
         <v>319</v>

</xml_diff>

<commit_message>
Aligned animal product demand with statistics by changing import, consumptions and prod system shares
</commit_message>
<xml_diff>
--- a/data/prod_parameters/DemandAndConversions.xlsx
+++ b/data/prod_parameters/DemandAndConversions.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1596" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="342">
   <si>
     <t>parameter</t>
   </si>
@@ -1077,7 +1077,19 @@
     <t>eggs</t>
   </si>
   <si>
-    <t>"Ägg"</t>
+    <t>Adjusted to match slaughter statistics</t>
+  </si>
+  <si>
+    <t>adj factor:</t>
+  </si>
+  <si>
+    <t>Adjusted to match egg prod. statistics</t>
+  </si>
+  <si>
+    <t>Adjusted to match prod. statistics. "Ägg"</t>
+  </si>
+  <si>
+    <t>CHECK THIS! Should be wheat distillers grain???</t>
   </si>
 </sst>
 </file>
@@ -1197,7 +1209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1241,6 +1253,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2645,11 +2660,14 @@
       <c r="J61" t="s">
         <v>18</v>
       </c>
-      <c r="K61">
-        <v>29.3</v>
+      <c r="K61" s="6">
+        <v>33.5</v>
       </c>
       <c r="L61" t="s">
         <v>19</v>
+      </c>
+      <c r="M61" s="6" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
@@ -4673,8 +4691,12 @@
       <c r="I180" s="4"/>
       <c r="J180" s="5"/>
       <c r="K180" s="5"/>
-      <c r="L180" s="5"/>
-      <c r="M180" s="5"/>
+      <c r="L180" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="M180" s="41">
+        <v>0.81799999999999995</v>
+      </c>
       <c r="N180" s="5"/>
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.25">
@@ -4685,8 +4707,8 @@
         <v>40</v>
       </c>
       <c r="K181" s="13">
-        <f>8.5*20/(29.5+8.5)</f>
-        <v>4.4736842105263159</v>
+        <f>8.5*20/(29.5+8.5)*$M$180</f>
+        <v>3.6594736842105262</v>
       </c>
       <c r="L181" t="s">
         <v>38</v>
@@ -4700,8 +4722,8 @@
         <v>40</v>
       </c>
       <c r="K182" s="13">
-        <f>(80.7*0+14.4*20+0.3*5*0)/(80.7+14.4+0.3*5)</f>
-        <v>2.981366459627329</v>
+        <f>(80.7*0+14.4*20+0.3*5*0)/(80.7+14.4+0.3*5)*$M$180</f>
+        <v>2.438757763975155</v>
       </c>
       <c r="L182" t="s">
         <v>38</v>
@@ -4715,8 +4737,8 @@
         <v>40</v>
       </c>
       <c r="K183" s="13">
-        <f>(45.6*0+44.1*20+1.3*5*0+1.8*10*0)/(45.6+44.1+1.3*5+1.8*10)</f>
-        <v>7.723292469352014</v>
+        <f>(45.6*0+44.1*20+1.3*5*0+1.8*10*0)/(45.6+44.1+1.3*5+1.8*10)*$M$180</f>
+        <v>6.317653239929947</v>
       </c>
       <c r="L183" t="s">
         <v>38</v>
@@ -4730,8 +4752,8 @@
         <v>40</v>
       </c>
       <c r="K184">
-        <f>60</f>
-        <v>60</v>
+        <f>60*$M$180</f>
+        <v>49.08</v>
       </c>
       <c r="L184" t="s">
         <v>38</v>
@@ -4745,6 +4767,7 @@
         <v>40</v>
       </c>
       <c r="K185">
+        <f>0*$M$180</f>
         <v>0</v>
       </c>
       <c r="L185" t="s">
@@ -4759,7 +4782,8 @@
         <v>40</v>
       </c>
       <c r="K186">
-        <v>20</v>
+        <f>20*$M$180</f>
+        <v>16.36</v>
       </c>
       <c r="L186" t="s">
         <v>38</v>
@@ -4773,7 +4797,8 @@
         <v>40</v>
       </c>
       <c r="K187">
-        <v>20</v>
+        <f>20*$M$180</f>
+        <v>16.36</v>
       </c>
       <c r="L187" t="s">
         <v>38</v>
@@ -4787,7 +4812,8 @@
         <v>40</v>
       </c>
       <c r="K188">
-        <v>20</v>
+        <f>20*$M$180</f>
+        <v>16.36</v>
       </c>
       <c r="L188" t="s">
         <v>38</v>
@@ -4801,8 +4827,8 @@
         <v>40</v>
       </c>
       <c r="K189">
-        <f>43</f>
-        <v>43</v>
+        <f>43*$M$180</f>
+        <v>35.173999999999999</v>
       </c>
       <c r="L189" t="s">
         <v>38</v>
@@ -4833,11 +4859,14 @@
       <c r="J191" t="s">
         <v>40</v>
       </c>
-      <c r="K191">
-        <v>37</v>
+      <c r="K191" s="6">
+        <v>37.5</v>
       </c>
       <c r="L191" t="s">
         <v>38</v>
+      </c>
+      <c r="M191" s="6" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
@@ -4847,11 +4876,14 @@
       <c r="J192" t="s">
         <v>40</v>
       </c>
-      <c r="K192" s="17">
-        <v>43</v>
+      <c r="K192" s="6">
+        <v>48.1</v>
       </c>
       <c r="L192" t="s">
         <v>38</v>
+      </c>
+      <c r="M192" s="6" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
@@ -4861,11 +4893,14 @@
       <c r="J193" t="s">
         <v>40</v>
       </c>
-      <c r="K193" s="17">
-        <v>36</v>
+      <c r="K193" s="6">
+        <v>46.1</v>
       </c>
       <c r="L193" t="s">
         <v>38</v>
+      </c>
+      <c r="M193" s="6" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
@@ -4893,11 +4928,14 @@
       <c r="J195" t="s">
         <v>40</v>
       </c>
-      <c r="K195" s="17">
-        <v>12</v>
+      <c r="K195" s="6">
+        <v>10</v>
       </c>
       <c r="L195" t="s">
         <v>38</v>
+      </c>
+      <c r="M195" s="6" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
@@ -5905,8 +5943,8 @@
       <c r="J246" t="s">
         <v>41</v>
       </c>
-      <c r="K246" s="15">
-        <v>17</v>
+      <c r="K246" s="29">
+        <v>15.75</v>
       </c>
       <c r="L246" t="s">
         <v>38</v>
@@ -5950,10 +5988,13 @@
         <v>41</v>
       </c>
       <c r="K248" s="6">
-        <v>2.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="L248" t="s">
         <v>38</v>
+      </c>
+      <c r="M248" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="249" spans="1:14" x14ac:dyDescent="0.25">
@@ -5970,10 +6011,13 @@
         <v>41</v>
       </c>
       <c r="K249" s="6">
-        <v>15.4</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="L249" t="s">
         <v>38</v>
+      </c>
+      <c r="M249" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="250" spans="1:14" x14ac:dyDescent="0.25">
@@ -5990,10 +6034,13 @@
         <v>41</v>
       </c>
       <c r="K250" s="6">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="L250" t="s">
         <v>38</v>
+      </c>
+      <c r="M250" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="251" spans="1:14" x14ac:dyDescent="0.25">
@@ -6027,14 +6074,14 @@
       <c r="J252" t="s">
         <v>41</v>
       </c>
-      <c r="K252" s="17">
-        <v>19.399999999999999</v>
+      <c r="K252" s="6">
+        <v>16.5</v>
       </c>
       <c r="L252" t="s">
         <v>38</v>
       </c>
-      <c r="M252" t="s">
-        <v>337</v>
+      <c r="M252" s="6" t="s">
+        <v>340</v>
       </c>
       <c r="N252" s="26" t="s">
         <v>222</v>
@@ -8984,17 +9031,19 @@
       <c r="G375" s="10"/>
       <c r="H375" s="10"/>
       <c r="I375" s="10"/>
-      <c r="J375" t="s">
+      <c r="J375" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="K375" s="20">
+      <c r="K375" s="12">
         <v>11</v>
       </c>
-      <c r="L375" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="M375" s="8"/>
-      <c r="N375" s="8" t="s">
+      <c r="L375" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="M375" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="N375" s="10" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Various updates to parameter sheets
</commit_message>
<xml_diff>
--- a/data/prod_parameters/DemandAndConversions.xlsx
+++ b/data/prod_parameters/DemandAndConversions.xlsx
@@ -10,8 +10,9 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
     <sheet name="Trade" sheetId="4" r:id="rId3"/>
+    <sheet name="references" sheetId="5" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1620" uniqueCount="356">
   <si>
     <t>parameter</t>
   </si>
@@ -398,9 +399,6 @@
     <t>rye bran</t>
   </si>
   <si>
-    <t>oat offals</t>
-  </si>
-  <si>
     <t>potatoe offals</t>
   </si>
   <si>
@@ -743,28 +741,6 @@
     <t>sugar beet</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Higher factor for syrup than sugar?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Assumed from sugar beet for domestic prod</t>
-    </r>
-  </si>
-  <si>
     <t>sugar beet pulp</t>
   </si>
   <si>
@@ -1038,18 +1014,12 @@
     <t>Börjesson, P., Tufvesson, L., &amp; Lantz, M. (2010). Livscykelanalys av svenska biodrivmedel. (Environmental and Energy System Studies report no. 70; Vol. 70). Environmental and Energy Systems Studies, Lund university.</t>
   </si>
   <si>
-    <t>2.1 kg DM wheat --&gt; 1 L bioethanol + 0.8 kg DM distillers grain. Wheat 86% DM, distillers grain 11% DM. Bioethanol 21.3 MJ/L and 27.8 MJ/kg --&gt; 0.8 kg/L</t>
-  </si>
-  <si>
     <t>PROCESSING ENERGY USE</t>
   </si>
   <si>
     <t>Add processing energy use factors per food item</t>
   </si>
   <si>
-    <t>Baseds on assuming 600 000 tonnes cereals used</t>
-  </si>
-  <si>
     <t>Rice and products, refined</t>
   </si>
   <si>
@@ -1090,6 +1060,60 @@
   </si>
   <si>
     <t>CHECK THIS! Should be wheat distillers grain???</t>
+  </si>
+  <si>
+    <t>@ 90% DM</t>
+  </si>
+  <si>
+    <t>Tabell A18 in Börjesson et al (2010)</t>
+  </si>
+  <si>
+    <t>Börjesson et al (2010)</t>
+  </si>
+  <si>
+    <t>Based on assuming 600 000 tonnes cereals used</t>
+  </si>
+  <si>
+    <t>2.1 kg DM wheat --&gt; 1 L bioethanol + 0.8 kg DM distillers grain. Wheat 86% DM, distillers grain 90% DM. Bioethanol 21.3 MJ/L and 27.8 MJ/kg --&gt; 0.766 kg/L</t>
+  </si>
+  <si>
+    <t>havrekli??</t>
+  </si>
+  <si>
+    <t>oat bran</t>
+  </si>
+  <si>
+    <t>161 kg WS/t SB</t>
+  </si>
+  <si>
+    <t>Garcia Gonzalez, M. N., &amp; Björnsson, L. (2022). Life cycle assessment of the production of beet sugar and its by-products. Journal of Cleaner Production, 346, 131211. doi:https://doi.org/10.1016/j.jclepro.2022.131211</t>
+  </si>
+  <si>
+    <t>Garcia Gonzalez and Börjesson 2022</t>
+  </si>
+  <si>
+    <t>(90% DM) 6.4 kg DM PSBP and 25.2 kg DM DSBP per t wet weight sugar beet</t>
+  </si>
+  <si>
+    <t>(76% DM) 19 kg DM molasses per t wet weight sugar beet</t>
+  </si>
+  <si>
+    <t>Based on sugar but adjusted to 20% w.c. in syrup</t>
+  </si>
+  <si>
+    <t>https://fransverige.se/aktuellt/nya-siffror-visar-sveriges-sjalvforsorjningsgrad/</t>
+  </si>
+  <si>
+    <t>43.6% 2019. Adjusted to match slaughter statistics</t>
+  </si>
+  <si>
+    <t>23.3% 2019. Adjusted to match slaughter statistics</t>
+  </si>
+  <si>
+    <t>28.4% 2019. Adjusted to match slaughter statistics</t>
+  </si>
+  <si>
+    <t>for 2019</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1233,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1256,6 +1280,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1669,7 +1695,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
@@ -1685,15 +1711,15 @@
         <v>19</v>
       </c>
       <c r="M7" s="17" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="N7" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B8" t="s">
         <v>26</v>
@@ -1711,7 +1737,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
@@ -1727,15 +1753,15 @@
         <v>19</v>
       </c>
       <c r="M9" s="17" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="N9" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -1754,7 +1780,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
@@ -1770,12 +1796,12 @@
         <v>19</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
@@ -1811,7 +1837,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B14" t="s">
         <v>26</v>
@@ -1827,12 +1853,12 @@
         <v>19</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
@@ -1851,7 +1877,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s">
         <v>26</v>
@@ -1867,12 +1893,12 @@
         <v>19</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B17" t="s">
         <v>26</v>
@@ -1891,7 +1917,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
@@ -1907,12 +1933,12 @@
         <v>19</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -1983,7 +2009,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B23" t="s">
         <v>103</v>
@@ -2020,7 +2046,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2038,7 +2064,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B26" t="s">
         <v>108</v>
@@ -2055,7 +2081,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B27" t="s">
         <v>108</v>
@@ -2072,7 +2098,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B28" t="s">
         <v>108</v>
@@ -2089,7 +2115,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B29" t="s">
         <v>108</v>
@@ -2106,7 +2132,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B30" t="s">
         <v>108</v>
@@ -2123,7 +2149,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B31" t="s">
         <v>108</v>
@@ -2174,7 +2200,7 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B34" t="s">
         <v>108</v>
@@ -2191,7 +2217,7 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B35" t="s">
         <v>108</v>
@@ -2207,7 +2233,7 @@
         <v>19</v>
       </c>
       <c r="M35" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -2216,7 +2242,7 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2234,10 +2260,10 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B38" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J38" t="s">
         <v>18</v>
@@ -2251,10 +2277,10 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="B39" t="s">
         <v>250</v>
-      </c>
-      <c r="B39" t="s">
-        <v>252</v>
       </c>
       <c r="J39" t="s">
         <v>18</v>
@@ -2268,10 +2294,10 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B40" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J40" t="s">
         <v>18</v>
@@ -2285,10 +2311,10 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="17" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B41" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J41" t="s">
         <v>18</v>
@@ -2302,10 +2328,10 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B42" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J42" t="s">
         <v>18</v>
@@ -2318,15 +2344,15 @@
         <v>19</v>
       </c>
       <c r="M42" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B43" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J43" t="s">
         <v>18</v>
@@ -2340,10 +2366,10 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B44" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C44" s="9"/>
       <c r="J44" t="s">
@@ -2356,15 +2382,15 @@
         <v>19</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B45" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="J45" t="s">
         <v>18</v>
@@ -2377,7 +2403,7 @@
         <v>19</v>
       </c>
       <c r="M45" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -2617,7 +2643,7 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B59" t="s">
         <v>55</v>
@@ -2655,19 +2681,20 @@
         <v>15</v>
       </c>
       <c r="B61" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="J61" t="s">
         <v>18</v>
       </c>
       <c r="K61" s="6">
-        <v>33.5</v>
+        <f>29.3+1.6</f>
+        <v>30.900000000000002</v>
       </c>
       <c r="L61" t="s">
         <v>19</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
@@ -2708,10 +2735,10 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B64" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J64" t="s">
         <v>18</v>
@@ -2725,10 +2752,10 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B65" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J65" t="s">
         <v>18</v>
@@ -2742,10 +2769,10 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B66" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J66" t="s">
         <v>18</v>
@@ -2759,10 +2786,10 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B67" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J67" t="s">
         <v>18</v>
@@ -2776,10 +2803,10 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="26" t="s">
+        <v>212</v>
+      </c>
+      <c r="B68" t="s">
         <v>213</v>
-      </c>
-      <c r="B68" t="s">
-        <v>214</v>
       </c>
       <c r="J68" t="s">
         <v>18</v>
@@ -2829,10 +2856,10 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>131</v>
+      </c>
+      <c r="B71" t="s">
         <v>132</v>
-      </c>
-      <c r="B71" t="s">
-        <v>133</v>
       </c>
       <c r="J71" t="s">
         <v>18</v>
@@ -2845,15 +2872,15 @@
         <v>19</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B72" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J72" t="s">
         <v>18</v>
@@ -2866,15 +2893,15 @@
         <v>19</v>
       </c>
       <c r="M72" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B73" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J73" t="s">
         <v>18</v>
@@ -2887,7 +2914,7 @@
         <v>19</v>
       </c>
       <c r="M73" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -2910,10 +2937,10 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B75" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J75" t="s">
         <v>18</v>
@@ -2927,10 +2954,10 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>225</v>
+      </c>
+      <c r="B76" t="s">
         <v>226</v>
-      </c>
-      <c r="B76" t="s">
-        <v>227</v>
       </c>
       <c r="J76" t="s">
         <v>18</v>
@@ -2942,15 +2969,15 @@
         <v>19</v>
       </c>
       <c r="M76" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B77" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J77" t="s">
         <v>18</v>
@@ -2982,7 +3009,7 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B79" t="s">
         <v>112</v>
@@ -2999,7 +3026,7 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B80" t="s">
         <v>112</v>
@@ -3016,7 +3043,7 @@
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B81" t="s">
         <v>112</v>
@@ -3031,12 +3058,12 @@
         <v>19</v>
       </c>
       <c r="M81" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B82" t="s">
         <v>112</v>
@@ -3051,7 +3078,7 @@
         <v>19</v>
       </c>
       <c r="M82" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.25">
@@ -3128,7 +3155,7 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -3146,48 +3173,50 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B89" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H89" t="s">
         <v>45</v>
       </c>
       <c r="J89" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K89" s="33">
-        <v>197000</v>
+        <f>600000*(K379/100)</f>
+        <v>188217.14285714284</v>
       </c>
       <c r="L89" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M89" s="17" t="s">
-        <v>327</v>
-      </c>
+        <v>341</v>
+      </c>
+      <c r="N89" s="21"/>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B90" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H90" t="s">
         <v>45</v>
       </c>
       <c r="J90" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K90" s="33">
         <v>10000</v>
       </c>
       <c r="L90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M90" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -3198,25 +3227,25 @@
         <v>101</v>
       </c>
       <c r="B92" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H92" t="s">
         <v>45</v>
       </c>
       <c r="J92" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K92" s="33">
         <v>34000</v>
       </c>
       <c r="L92" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M92" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="N92" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
@@ -3224,25 +3253,25 @@
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B94" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H94" t="s">
         <v>45</v>
       </c>
       <c r="J94" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K94" s="37">
         <v>355.5</v>
       </c>
       <c r="L94" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="M94" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
@@ -3250,7 +3279,7 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -3268,132 +3297,132 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B97" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H97" t="s">
         <v>45</v>
       </c>
       <c r="J97" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K97" s="33">
         <v>558249.80000000005</v>
       </c>
       <c r="L97" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M97" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="N97" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B98" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H98" t="s">
         <v>45</v>
       </c>
       <c r="J98" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K98" s="33">
         <v>304650.40000000002</v>
       </c>
       <c r="L98" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M98" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="N98" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>297</v>
+      </c>
+      <c r="B99" t="s">
         <v>299</v>
-      </c>
-      <c r="B99" t="s">
-        <v>301</v>
       </c>
       <c r="H99" t="s">
         <v>45</v>
       </c>
       <c r="J99" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K99" s="33">
         <v>32965.800000000003</v>
       </c>
       <c r="L99" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M99" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="N99" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B100" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H100" t="s">
         <v>45</v>
       </c>
       <c r="J100" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K100" s="33">
         <v>177249.6</v>
       </c>
       <c r="L100" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M100" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="N100" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B101" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H101" t="s">
         <v>45</v>
       </c>
       <c r="J101" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K101" s="33">
         <v>22062.799999999999</v>
       </c>
       <c r="L101" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M101" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="N101" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
@@ -3401,25 +3430,25 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H102" t="s">
         <v>45</v>
       </c>
       <c r="J102" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K102" s="33">
         <v>25000</v>
       </c>
       <c r="L102" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M102" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="N102" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.25">
@@ -3604,7 +3633,7 @@
     </row>
     <row r="114" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I114" t="s">
         <v>50</v>
@@ -3621,7 +3650,7 @@
     </row>
     <row r="115" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I115" t="s">
         <v>51</v>
@@ -3638,7 +3667,7 @@
     </row>
     <row r="116" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I116" t="s">
         <v>52</v>
@@ -3767,7 +3796,7 @@
     </row>
     <row r="123" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="I123" t="s">
         <v>50</v>
@@ -3784,7 +3813,7 @@
     </row>
     <row r="124" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B124" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="I124" t="s">
         <v>51</v>
@@ -3801,7 +3830,7 @@
     </row>
     <row r="125" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B125" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="I125" t="s">
         <v>52</v>
@@ -3821,7 +3850,7 @@
     </row>
     <row r="126" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I126" t="s">
         <v>50</v>
@@ -3838,7 +3867,7 @@
     </row>
     <row r="127" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I127" t="s">
         <v>51</v>
@@ -3855,7 +3884,7 @@
     </row>
     <row r="128" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I128" t="s">
         <v>52</v>
@@ -3875,7 +3904,7 @@
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I129" t="s">
         <v>50</v>
@@ -3892,7 +3921,7 @@
     </row>
     <row r="130" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I130" t="s">
         <v>51</v>
@@ -3909,7 +3938,7 @@
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I131" t="s">
         <v>52</v>
@@ -3929,7 +3958,7 @@
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I132" t="s">
         <v>50</v>
@@ -3946,7 +3975,7 @@
     </row>
     <row r="133" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I133" t="s">
         <v>51</v>
@@ -3963,7 +3992,7 @@
     </row>
     <row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I134" t="s">
         <v>52</v>
@@ -4091,7 +4120,7 @@
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J142" t="s">
         <v>40</v>
@@ -4105,7 +4134,7 @@
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J143" t="s">
         <v>40</v>
@@ -4118,12 +4147,12 @@
         <v>38</v>
       </c>
       <c r="M143" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="144" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="J144" t="s">
         <v>40</v>
@@ -4137,7 +4166,7 @@
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="J145" t="s">
         <v>40</v>
@@ -4150,12 +4179,12 @@
         <v>38</v>
       </c>
       <c r="M145" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="J146" t="s">
         <v>40</v>
@@ -4169,7 +4198,7 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J147" t="s">
         <v>40</v>
@@ -4182,7 +4211,7 @@
         <v>38</v>
       </c>
       <c r="M147" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.25">
@@ -4201,7 +4230,7 @@
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J149" t="s">
         <v>40</v>
@@ -4215,7 +4244,7 @@
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J150" t="s">
         <v>40</v>
@@ -4228,12 +4257,12 @@
         <v>38</v>
       </c>
       <c r="M150" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J151" t="s">
         <v>40</v>
@@ -4247,7 +4276,7 @@
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J152" t="s">
         <v>40</v>
@@ -4260,12 +4289,12 @@
         <v>38</v>
       </c>
       <c r="M152" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J153" t="s">
         <v>40</v>
@@ -4277,12 +4306,12 @@
         <v>38</v>
       </c>
       <c r="M153" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="J154" t="s">
         <v>40</v>
@@ -4295,7 +4324,7 @@
         <v>38</v>
       </c>
       <c r="M154" s="27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.25">
@@ -4346,7 +4375,7 @@
     </row>
     <row r="158" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A158" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J158" t="s">
         <v>40</v>
@@ -4392,7 +4421,7 @@
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="J161" t="s">
         <v>40</v>
@@ -4406,7 +4435,7 @@
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="17" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="J162" t="s">
         <v>40</v>
@@ -4420,7 +4449,7 @@
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A163" s="17" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="J163" t="s">
         <v>40</v>
@@ -4434,7 +4463,7 @@
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A164" s="17" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="J164" t="s">
         <v>40</v>
@@ -4448,7 +4477,7 @@
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="17" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="J165" t="s">
         <v>40</v>
@@ -4460,12 +4489,12 @@
         <v>38</v>
       </c>
       <c r="M165" s="6" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="J166" t="s">
         <v>40</v>
@@ -4479,7 +4508,7 @@
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C167" s="9"/>
       <c r="J167" t="s">
@@ -4492,12 +4521,12 @@
         <v>38</v>
       </c>
       <c r="M167" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="17" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="J168" t="s">
         <v>40</v>
@@ -4509,7 +4538,7 @@
         <v>38</v>
       </c>
       <c r="M168" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.25">
@@ -4532,7 +4561,7 @@
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J170" t="s">
         <v>40</v>
@@ -4546,7 +4575,7 @@
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J171" t="s">
         <v>40</v>
@@ -4560,7 +4589,7 @@
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J172" t="s">
         <v>40</v>
@@ -4574,7 +4603,7 @@
     </row>
     <row r="173" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A173" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J173" t="s">
         <v>40</v>
@@ -4589,7 +4618,7 @@
     </row>
     <row r="174" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A174" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J174" t="s">
         <v>40</v>
@@ -4601,12 +4630,12 @@
         <v>38</v>
       </c>
       <c r="M174" s="6" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="175" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A175" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J175" t="s">
         <v>40</v>
@@ -4648,7 +4677,7 @@
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A178" s="17" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="J178" t="s">
         <v>40</v>
@@ -4662,7 +4691,7 @@
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A179" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J179" t="s">
         <v>40</v>
@@ -4674,7 +4703,7 @@
         <v>38</v>
       </c>
       <c r="M179" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.25">
@@ -4692,7 +4721,7 @@
       <c r="J180" s="5"/>
       <c r="K180" s="5"/>
       <c r="L180" s="5" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="M180" s="41">
         <v>0.81799999999999995</v>
@@ -4866,7 +4895,10 @@
         <v>38</v>
       </c>
       <c r="M191" s="6" t="s">
-        <v>337</v>
+        <v>353</v>
+      </c>
+      <c r="N191" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
@@ -4883,12 +4915,15 @@
         <v>38</v>
       </c>
       <c r="M192" s="6" t="s">
-        <v>337</v>
+        <v>352</v>
+      </c>
+      <c r="N192" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="J193" t="s">
         <v>40</v>
@@ -4900,7 +4935,10 @@
         <v>38</v>
       </c>
       <c r="M193" s="6" t="s">
-        <v>337</v>
+        <v>354</v>
+      </c>
+      <c r="N193" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
@@ -4928,14 +4966,18 @@
       <c r="J195" t="s">
         <v>40</v>
       </c>
-      <c r="K195" s="6">
-        <v>10</v>
+      <c r="K195" s="17">
+        <f>2.5</f>
+        <v>2.5</v>
       </c>
       <c r="L195" t="s">
         <v>38</v>
       </c>
-      <c r="M195" s="6" t="s">
-        <v>339</v>
+      <c r="M195" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="N195" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
@@ -4958,7 +5000,7 @@
     </row>
     <row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J197" t="s">
         <v>40</v>
@@ -4972,7 +5014,7 @@
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A198" s="26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="J198" t="s">
         <v>40</v>
@@ -4986,7 +5028,7 @@
     </row>
     <row r="199" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A199" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J199" t="s">
         <v>40</v>
@@ -4998,12 +5040,12 @@
         <v>38</v>
       </c>
       <c r="M199" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="200" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A200" s="26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J200" t="s">
         <v>40</v>
@@ -5017,7 +5059,7 @@
     </row>
     <row r="201" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A201" s="26" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B201" s="8"/>
       <c r="C201" s="8"/>
@@ -5059,7 +5101,7 @@
     </row>
     <row r="203" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J203" t="s">
         <v>40</v>
@@ -5092,7 +5134,7 @@
     </row>
     <row r="205" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J205" t="s">
         <v>40</v>
@@ -5104,12 +5146,12 @@
         <v>38</v>
       </c>
       <c r="M205" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J206" t="s">
         <v>40</v>
@@ -5122,12 +5164,12 @@
         <v>38</v>
       </c>
       <c r="M206" s="27" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J207" t="s">
         <v>40</v>
@@ -5159,7 +5201,7 @@
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="J209" t="s">
         <v>40</v>
@@ -5173,7 +5215,7 @@
     </row>
     <row r="210" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J210" t="s">
         <v>40</v>
@@ -5190,7 +5232,7 @@
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="J211" t="s">
         <v>40</v>
@@ -5202,12 +5244,12 @@
         <v>38</v>
       </c>
       <c r="M211" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="212" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="J212" t="s">
         <v>40</v>
@@ -5219,12 +5261,12 @@
         <v>38</v>
       </c>
       <c r="M212" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B214" s="2"/>
       <c r="C214" s="2"/>
@@ -5256,7 +5298,7 @@
         <v>46</v>
       </c>
       <c r="M215" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="216" spans="1:14" x14ac:dyDescent="0.25">
@@ -5298,7 +5340,7 @@
     </row>
     <row r="218" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G218" t="s">
         <v>87</v>
@@ -5316,7 +5358,7 @@
         <v>38</v>
       </c>
       <c r="M218" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N218" t="s">
         <v>98</v>
@@ -5324,7 +5366,7 @@
     </row>
     <row r="219" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G219" t="s">
         <v>87</v>
@@ -5345,7 +5387,7 @@
     </row>
     <row r="220" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G220" t="s">
         <v>87</v>
@@ -5363,7 +5405,7 @@
         <v>38</v>
       </c>
       <c r="M220" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N220" t="s">
         <v>98</v>
@@ -5371,7 +5413,7 @@
     </row>
     <row r="221" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G221" t="s">
         <v>87</v>
@@ -5392,7 +5434,7 @@
     </row>
     <row r="222" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G222" t="s">
         <v>87</v>
@@ -5410,7 +5452,7 @@
         <v>38</v>
       </c>
       <c r="M222" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N222" t="s">
         <v>98</v>
@@ -5418,7 +5460,7 @@
     </row>
     <row r="223" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G223" t="s">
         <v>87</v>
@@ -5439,7 +5481,7 @@
     </row>
     <row r="224" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G224" t="s">
         <v>87</v>
@@ -5457,15 +5499,15 @@
         <v>38</v>
       </c>
       <c r="M224" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="N224" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="225" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G225" t="s">
         <v>87</v>
@@ -5487,7 +5529,7 @@
     </row>
     <row r="226" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G226" t="s">
         <v>87</v>
@@ -5507,7 +5549,7 @@
     </row>
     <row r="227" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G227" t="s">
         <v>87</v>
@@ -5564,7 +5606,7 @@
         <v>38</v>
       </c>
       <c r="N229" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="230" spans="1:14" x14ac:dyDescent="0.25">
@@ -5587,12 +5629,12 @@
         <v>38</v>
       </c>
       <c r="N230" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="231" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A231" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G231" t="s">
         <v>87</v>
@@ -5650,7 +5692,7 @@
     </row>
     <row r="234" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A234" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G234" t="s">
         <v>87</v>
@@ -5668,15 +5710,15 @@
         <v>38</v>
       </c>
       <c r="M234" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="N234" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="235" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A235" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G235" t="s">
         <v>87</v>
@@ -5694,15 +5736,15 @@
         <v>38</v>
       </c>
       <c r="M235" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N235" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="236" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A236" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G236" t="s">
         <v>87</v>
@@ -5720,10 +5762,10 @@
         <v>38</v>
       </c>
       <c r="M236" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N236" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="237" spans="1:14" x14ac:dyDescent="0.25">
@@ -5746,10 +5788,10 @@
         <v>38</v>
       </c>
       <c r="M237" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N237" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="238" spans="1:14" x14ac:dyDescent="0.25">
@@ -5772,15 +5814,15 @@
         <v>38</v>
       </c>
       <c r="M238" s="26" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N238" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="239" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A239" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G239" t="s">
         <v>87</v>
@@ -5821,7 +5863,7 @@
     </row>
     <row r="241" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A241" s="17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H241" t="s">
         <v>43</v>
@@ -5836,15 +5878,15 @@
         <v>38</v>
       </c>
       <c r="M241" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="N241" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="242" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A242" s="17" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H242" t="s">
         <v>43</v>
@@ -5859,15 +5901,15 @@
         <v>38</v>
       </c>
       <c r="M242" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="N242" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="243" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A243" s="17" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H243" t="s">
         <v>43</v>
@@ -5882,15 +5924,15 @@
         <v>38</v>
       </c>
       <c r="M243" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="N243" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="244" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A244" s="17" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H244" t="s">
         <v>43</v>
@@ -5905,10 +5947,10 @@
         <v>38</v>
       </c>
       <c r="M244" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="N244" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="245" spans="1:14" x14ac:dyDescent="0.25">
@@ -5950,7 +5992,7 @@
         <v>38</v>
       </c>
       <c r="M246" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N246" t="s">
         <v>94</v>
@@ -5994,7 +6036,7 @@
         <v>38</v>
       </c>
       <c r="M248" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="249" spans="1:14" x14ac:dyDescent="0.25">
@@ -6017,12 +6059,12 @@
         <v>38</v>
       </c>
       <c r="M249" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="250" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="G250" t="s">
         <v>87</v>
@@ -6040,7 +6082,7 @@
         <v>38</v>
       </c>
       <c r="M250" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="251" spans="1:14" x14ac:dyDescent="0.25">
@@ -6081,10 +6123,10 @@
         <v>38</v>
       </c>
       <c r="M252" s="6" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="N252" s="26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="253" spans="1:14" x14ac:dyDescent="0.25">
@@ -6107,7 +6149,7 @@
     </row>
     <row r="254" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B254" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H254" t="s">
         <v>43</v>
@@ -6122,10 +6164,10 @@
         <v>38</v>
       </c>
       <c r="M254" t="s">
+        <v>220</v>
+      </c>
+      <c r="N254" s="26" t="s">
         <v>221</v>
-      </c>
-      <c r="N254" s="26" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="255" spans="1:14" x14ac:dyDescent="0.25">
@@ -6148,7 +6190,7 @@
     </row>
     <row r="256" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G256" t="s">
         <v>87</v>
@@ -6186,7 +6228,7 @@
     </row>
     <row r="258" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H258" t="s">
         <v>43</v>
@@ -6201,15 +6243,15 @@
         <v>38</v>
       </c>
       <c r="M258" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="N258" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="259" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H259" t="s">
         <v>43</v>
@@ -6224,15 +6266,15 @@
         <v>38</v>
       </c>
       <c r="M259" t="s">
+        <v>171</v>
+      </c>
+      <c r="N259" s="26" t="s">
         <v>172</v>
-      </c>
-      <c r="N259" s="26" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="260" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H260" t="s">
         <v>43</v>
@@ -6247,15 +6289,15 @@
         <v>38</v>
       </c>
       <c r="M260" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="N260" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="261" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H261" t="s">
         <v>43</v>
@@ -6270,10 +6312,10 @@
         <v>38</v>
       </c>
       <c r="M261" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="N261" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="264" spans="1:14" x14ac:dyDescent="0.25">
@@ -6342,7 +6384,7 @@
     </row>
     <row r="268" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C268" t="s">
         <v>37</v>
@@ -6362,7 +6404,7 @@
     </row>
     <row r="269" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C269" t="s">
         <v>37</v>
@@ -6385,7 +6427,7 @@
     </row>
     <row r="270" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C270" t="s">
         <v>37</v>
@@ -6408,7 +6450,7 @@
     </row>
     <row r="271" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C271" t="s">
         <v>37</v>
@@ -6428,7 +6470,7 @@
     </row>
     <row r="272" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A272" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B272" s="8"/>
       <c r="C272" s="8" t="s">
@@ -6456,7 +6498,7 @@
     </row>
     <row r="273" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A273" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B273" s="8"/>
       <c r="C273" s="8" t="s">
@@ -6486,7 +6528,7 @@
     </row>
     <row r="274" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A274" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B274" s="8"/>
       <c r="C274" s="8" t="s">
@@ -6516,7 +6558,7 @@
     </row>
     <row r="275" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A275" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B275" s="8"/>
       <c r="C275" s="8" t="s">
@@ -6544,7 +6586,7 @@
     </row>
     <row r="276" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A276" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B276" s="8"/>
       <c r="C276" s="8" t="s">
@@ -6574,7 +6616,7 @@
     </row>
     <row r="277" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B277" s="8"/>
       <c r="C277" s="9" t="s">
@@ -6602,7 +6644,7 @@
     </row>
     <row r="278" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B278" s="8"/>
       <c r="C278" s="9" t="s">
@@ -6632,7 +6674,7 @@
     </row>
     <row r="279" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B279" s="8"/>
       <c r="C279" s="9" t="s">
@@ -6660,7 +6702,7 @@
     </row>
     <row r="280" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B280" s="8"/>
       <c r="C280" s="9" t="s">
@@ -6688,7 +6730,7 @@
     </row>
     <row r="281" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B281" s="8"/>
       <c r="C281" s="9" t="s">
@@ -6697,7 +6739,7 @@
       <c r="D281" s="8"/>
       <c r="E281" s="8"/>
       <c r="F281" s="9" t="s">
-        <v>121</v>
+        <v>344</v>
       </c>
       <c r="G281" s="8"/>
       <c r="H281" s="8"/>
@@ -6711,14 +6753,16 @@
       <c r="L281" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="M281" s="8"/>
+      <c r="M281" s="10" t="s">
+        <v>343</v>
+      </c>
       <c r="N281" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="282" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B282" s="8"/>
       <c r="C282" s="9" t="s">
@@ -6727,7 +6771,7 @@
       <c r="D282" s="8"/>
       <c r="E282" s="8"/>
       <c r="F282" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G282" s="8"/>
       <c r="H282" s="8"/>
@@ -6748,7 +6792,7 @@
     </row>
     <row r="283" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B283" s="8"/>
       <c r="C283" s="9" t="s">
@@ -6776,7 +6820,7 @@
     </row>
     <row r="284" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B284" s="8"/>
       <c r="C284" s="9" t="s">
@@ -6785,7 +6829,7 @@
       <c r="D284" s="8"/>
       <c r="E284" s="8"/>
       <c r="F284" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G284" s="8"/>
       <c r="H284" s="8"/>
@@ -6806,7 +6850,7 @@
     </row>
     <row r="285" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B285" s="10"/>
       <c r="C285" s="9" t="s">
@@ -6828,13 +6872,13 @@
         <v>38</v>
       </c>
       <c r="M285" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="N285" s="8"/>
     </row>
     <row r="286" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B286" s="10"/>
       <c r="C286" s="8" t="s">
@@ -6856,13 +6900,13 @@
         <v>38</v>
       </c>
       <c r="M286" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="N286" s="8"/>
     </row>
     <row r="287" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B287" s="10"/>
       <c r="C287" s="9" t="s">
@@ -6884,13 +6928,13 @@
         <v>38</v>
       </c>
       <c r="M287" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="N287" s="8"/>
     </row>
     <row r="288" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B288" s="10"/>
       <c r="C288" s="9" t="s">
@@ -6912,7 +6956,7 @@
         <v>38</v>
       </c>
       <c r="M288" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="N288" s="8"/>
     </row>
@@ -6997,7 +7041,7 @@
       <c r="D292" s="8"/>
       <c r="E292" s="8"/>
       <c r="F292" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G292" s="8"/>
       <c r="H292" s="8"/>
@@ -7015,7 +7059,7 @@
     </row>
     <row r="293" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A293" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B293" s="8"/>
       <c r="C293" s="11" t="s">
@@ -7037,7 +7081,7 @@
         <v>38</v>
       </c>
       <c r="M293" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="294" spans="1:14" x14ac:dyDescent="0.25">
@@ -7076,7 +7120,7 @@
       <c r="D295" s="8"/>
       <c r="E295" s="8"/>
       <c r="F295" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G295" s="8"/>
       <c r="H295" s="8"/>
@@ -7092,10 +7136,10 @@
         <v>38</v>
       </c>
       <c r="M295" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="N295" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="N295" s="9" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="296" spans="1:14" x14ac:dyDescent="0.25">
@@ -7118,10 +7162,10 @@
     </row>
     <row r="297" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A297" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="C297" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="C297" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="J297" t="s">
         <v>85</v>
@@ -7135,10 +7179,10 @@
     </row>
     <row r="298" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A298" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C298" s="9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J298" t="s">
         <v>85</v>
@@ -7152,10 +7196,10 @@
     </row>
     <row r="299" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A299" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C299" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J299" t="s">
         <v>85</v>
@@ -7169,10 +7213,10 @@
     </row>
     <row r="300" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A300" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C300" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J300" t="s">
         <v>85</v>
@@ -7186,10 +7230,10 @@
     </row>
     <row r="301" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A301" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C301" s="9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J301" t="s">
         <v>85</v>
@@ -7203,10 +7247,10 @@
     </row>
     <row r="302" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C302" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J302" t="s">
         <v>85</v>
@@ -7270,11 +7314,11 @@
     </row>
     <row r="305" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A305" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B305" s="8"/>
       <c r="C305" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D305" s="8"/>
       <c r="E305" s="8"/>
@@ -7313,10 +7357,10 @@
     </row>
     <row r="307" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A307" s="17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C307" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J307" t="s">
         <v>85</v>
@@ -7330,10 +7374,10 @@
     </row>
     <row r="308" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" s="17" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C308" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J308" t="s">
         <v>85</v>
@@ -7350,13 +7394,13 @@
     </row>
     <row r="309" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A309" s="17" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C309" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F309" s="19" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J309" t="s">
         <v>86</v>
@@ -7373,10 +7417,10 @@
     </row>
     <row r="310" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A310" s="17" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C310" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J310" t="s">
         <v>85</v>
@@ -7393,13 +7437,13 @@
     </row>
     <row r="311" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A311" s="17" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C311" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="F311" s="19" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="J311" t="s">
         <v>86</v>
@@ -7416,10 +7460,10 @@
     </row>
     <row r="312" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A312" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="C312" s="9" t="s">
         <v>253</v>
-      </c>
-      <c r="C312" s="9" t="s">
-        <v>255</v>
       </c>
       <c r="J312" t="s">
         <v>85</v>
@@ -7433,10 +7477,10 @@
     </row>
     <row r="313" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A313" s="17" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C313" s="9" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="J313" t="s">
         <v>85</v>
@@ -7450,10 +7494,10 @@
     </row>
     <row r="314" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" s="17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C314" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="J314" t="s">
         <v>85</v>
@@ -7467,10 +7511,10 @@
     </row>
     <row r="315" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A315" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C315" s="9" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="J315" t="s">
         <v>85</v>
@@ -7484,10 +7528,10 @@
     </row>
     <row r="316" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A316" s="17" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C316" s="9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="J316" t="s">
         <v>85</v>
@@ -8070,7 +8114,7 @@
         <v>55</v>
       </c>
       <c r="F335" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G335" s="8"/>
       <c r="H335" s="8"/>
@@ -8105,7 +8149,7 @@
         <v>55</v>
       </c>
       <c r="F336" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G336" s="8"/>
       <c r="H336" s="8"/>
@@ -8140,7 +8184,7 @@
         <v>55</v>
       </c>
       <c r="F337" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G337" s="8"/>
       <c r="H337" s="8"/>
@@ -8175,7 +8219,7 @@
         <v>55</v>
       </c>
       <c r="F338" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G338" s="8"/>
       <c r="H338" s="8"/>
@@ -8237,7 +8281,7 @@
         <v>55</v>
       </c>
       <c r="F340" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G340" s="8"/>
       <c r="H340" s="8"/>
@@ -8272,7 +8316,7 @@
         <v>55</v>
       </c>
       <c r="F341" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G341" s="8"/>
       <c r="H341" s="8"/>
@@ -8307,7 +8351,7 @@
         <v>55</v>
       </c>
       <c r="F342" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G342" s="8"/>
       <c r="H342" s="8"/>
@@ -8342,7 +8386,7 @@
         <v>55</v>
       </c>
       <c r="F343" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G343" s="8"/>
       <c r="H343" s="8"/>
@@ -8363,12 +8407,12 @@
     </row>
     <row r="344" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B344" s="8"/>
       <c r="C344" s="8"/>
       <c r="D344" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E344" s="9" t="s">
         <v>55</v>
@@ -8391,18 +8435,18 @@
     </row>
     <row r="345" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A345" s="6" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B345" s="10"/>
       <c r="C345" s="10"/>
       <c r="D345" s="11" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E345" s="11" t="s">
         <v>55</v>
       </c>
       <c r="F345" s="11" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G345" s="8"/>
       <c r="H345" s="8"/>
@@ -8437,10 +8481,10 @@
       <c r="B347" s="8"/>
       <c r="C347" s="8"/>
       <c r="D347" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E347" s="9" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F347" s="8"/>
       <c r="G347" s="8"/>
@@ -8478,10 +8522,10 @@
     </row>
     <row r="349" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C349" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="J349" t="s">
         <v>85</v>
@@ -8495,10 +8539,10 @@
     </row>
     <row r="350" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A350" s="26" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C350" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J350" t="s">
         <v>85</v>
@@ -8512,10 +8556,10 @@
     </row>
     <row r="351" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A351" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C351" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J351" t="s">
         <v>85</v>
@@ -8529,12 +8573,12 @@
     </row>
     <row r="352" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A352" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="353" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A353" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B353" s="8"/>
       <c r="C353" s="8"/>
@@ -8567,10 +8611,10 @@
     </row>
     <row r="355" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C355" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H355" t="s">
         <v>45</v>
@@ -8591,13 +8635,13 @@
     </row>
     <row r="356" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C356" t="s">
+        <v>133</v>
+      </c>
+      <c r="F356" t="s">
         <v>134</v>
-      </c>
-      <c r="F356" t="s">
-        <v>135</v>
       </c>
       <c r="H356" t="s">
         <v>45</v>
@@ -8617,10 +8661,10 @@
     </row>
     <row r="357" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C357" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H357" t="s">
         <v>43</v>
@@ -8635,19 +8679,19 @@
         <v>38</v>
       </c>
       <c r="M357" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N357" s="8"/>
     </row>
     <row r="358" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C358" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F358" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H358" t="s">
         <v>43</v>
@@ -8683,96 +8727,119 @@
     </row>
     <row r="360" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C360" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J360" t="s">
         <v>85</v>
       </c>
-      <c r="K360" s="21">
-        <v>13</v>
+      <c r="K360" s="22">
+        <f>161/1000*100</f>
+        <v>16.100000000000001</v>
       </c>
       <c r="L360" t="s">
         <v>38</v>
+      </c>
+      <c r="M360" t="s">
+        <v>345</v>
+      </c>
+      <c r="N360" s="17" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="361" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C361" t="s">
+        <v>230</v>
+      </c>
+      <c r="F361" t="s">
         <v>231</v>
-      </c>
-      <c r="F361" t="s">
-        <v>233</v>
       </c>
       <c r="J361" t="s">
         <v>86</v>
       </c>
-      <c r="K361" s="21">
-        <v>7</v>
+      <c r="K361" s="22">
+        <f>(6.4+25.2)/1000/0.9*100</f>
+        <v>3.5111111111111115</v>
       </c>
       <c r="L361" t="s">
         <v>38</v>
+      </c>
+      <c r="M361" t="s">
+        <v>348</v>
+      </c>
+      <c r="N361" s="17" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="362" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C362" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F362" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="J362" t="s">
         <v>86</v>
       </c>
-      <c r="K362" s="21">
-        <v>4</v>
+      <c r="K362" s="22">
+        <f>19/1000/0.76*100</f>
+        <v>2.5</v>
       </c>
       <c r="L362" t="s">
         <v>38</v>
+      </c>
+      <c r="M362" t="s">
+        <v>349</v>
+      </c>
+      <c r="N362" s="17" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="363" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C363" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J363" t="s">
         <v>85</v>
       </c>
-      <c r="K363" s="23">
-        <v>13</v>
+      <c r="K363" s="43">
+        <f>K360/0.8</f>
+        <v>20.125</v>
       </c>
       <c r="L363" t="s">
         <v>38</v>
       </c>
-      <c r="M363" t="s">
-        <v>232</v>
+      <c r="M363" s="17" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="364" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C364" t="s">
+        <v>230</v>
+      </c>
+      <c r="F364" t="s">
         <v>231</v>
-      </c>
-      <c r="F364" t="s">
-        <v>233</v>
       </c>
       <c r="J364" t="s">
         <v>86</v>
       </c>
-      <c r="K364" s="21">
-        <v>7</v>
+      <c r="K364" s="43">
+        <f>K361</f>
+        <v>3.5111111111111115</v>
       </c>
       <c r="L364" t="s">
         <v>38</v>
@@ -8780,19 +8847,20 @@
     </row>
     <row r="365" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C365" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F365" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="J365" t="s">
         <v>86</v>
       </c>
-      <c r="K365" s="21">
-        <v>4</v>
+      <c r="K365" s="43">
+        <f>K362</f>
+        <v>2.5</v>
       </c>
       <c r="L365" t="s">
         <v>38</v>
@@ -8800,7 +8868,7 @@
     </row>
     <row r="366" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A366" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="367" spans="1:14" x14ac:dyDescent="0.25">
@@ -8823,11 +8891,11 @@
     </row>
     <row r="368" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B368" s="10"/>
       <c r="C368" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D368" s="10"/>
       <c r="E368" s="10"/>
@@ -8851,7 +8919,7 @@
     </row>
     <row r="369" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B369" s="10"/>
       <c r="C369" s="8" t="s">
@@ -8880,7 +8948,7 @@
     </row>
     <row r="370" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B370" s="10"/>
       <c r="C370" s="8" t="s">
@@ -8889,7 +8957,7 @@
       <c r="D370" s="10"/>
       <c r="E370" s="10"/>
       <c r="F370" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G370" s="10"/>
       <c r="H370" s="10"/>
@@ -8917,7 +8985,7 @@
       <c r="D371" s="10"/>
       <c r="E371" s="10"/>
       <c r="F371" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G371" s="10"/>
       <c r="H371" s="10"/>
@@ -8925,17 +8993,17 @@
       <c r="K371" s="20"/>
       <c r="L371" s="9"/>
       <c r="M371" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N371" s="8"/>
     </row>
     <row r="372" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B372" s="10"/>
       <c r="C372" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D372" s="10"/>
       <c r="E372" s="10"/>
@@ -8959,16 +9027,16 @@
     </row>
     <row r="373" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B373" s="10"/>
       <c r="C373" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D373" s="10"/>
       <c r="E373" s="10"/>
       <c r="F373" s="19" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="G373" s="10"/>
       <c r="H373" s="10"/>
@@ -8989,7 +9057,7 @@
     </row>
     <row r="374" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B374" s="10"/>
       <c r="C374" s="9" t="s">
@@ -9017,7 +9085,7 @@
     </row>
     <row r="375" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B375" s="10"/>
       <c r="C375" s="9" t="s">
@@ -9026,7 +9094,7 @@
       <c r="D375" s="10"/>
       <c r="E375" s="10"/>
       <c r="F375" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G375" s="10"/>
       <c r="H375" s="10"/>
@@ -9041,7 +9109,7 @@
         <v>38</v>
       </c>
       <c r="M375" s="10" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="N375" s="10" t="s">
         <v>92</v>
@@ -9049,7 +9117,7 @@
     </row>
     <row r="376" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A376" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B376" s="4"/>
       <c r="C376" s="4"/>
@@ -9067,11 +9135,11 @@
     </row>
     <row r="377" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B377" s="10"/>
       <c r="C377" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J377" t="s">
         <v>85</v>
@@ -9083,7 +9151,7 @@
         <v>38</v>
       </c>
       <c r="M377" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="N377" s="8" t="s">
         <v>92</v>
@@ -9091,14 +9159,14 @@
     </row>
     <row r="378" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B378" s="10"/>
       <c r="C378" t="s">
+        <v>133</v>
+      </c>
+      <c r="F378" t="s">
         <v>134</v>
-      </c>
-      <c r="F378" t="s">
-        <v>135</v>
       </c>
       <c r="J378" t="s">
         <v>86</v>
@@ -9115,7 +9183,7 @@
     </row>
     <row r="379" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A379" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B379" s="10"/>
       <c r="C379" t="s">
@@ -9125,59 +9193,63 @@
         <v>85</v>
       </c>
       <c r="K379" s="15">
-        <v>33</v>
+        <f>(1*0.766) / (2.1/0.86) * 100</f>
+        <v>31.369523809523809</v>
       </c>
       <c r="L379" s="17" t="s">
         <v>38</v>
       </c>
       <c r="M379" s="17" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="N379" s="9" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="380" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A380" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B380" s="10"/>
       <c r="C380" t="s">
         <v>37</v>
       </c>
       <c r="F380" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J380" t="s">
         <v>86</v>
       </c>
       <c r="K380" s="15">
-        <v>298</v>
+        <f>(0.8/0.9) / (2.1/0.86) * 100</f>
+        <v>36.402116402116405</v>
       </c>
       <c r="L380" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="M380" s="17"/>
+      <c r="M380" s="42" t="s">
+        <v>338</v>
+      </c>
       <c r="N380" s="9" t="s">
-        <v>323</v>
+        <v>340</v>
       </c>
     </row>
     <row r="381" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A381" s="6"/>
       <c r="B381" s="10"/>
       <c r="F381" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="K381" s="23"/>
       <c r="L381" s="6"/>
       <c r="M381" s="6" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="N381" s="9"/>
     </row>
     <row r="382" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A382" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B382" s="4"/>
       <c r="C382" s="4"/>
@@ -9189,7 +9261,7 @@
       <c r="I382" s="4"/>
       <c r="J382" s="5"/>
       <c r="K382" s="38" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="L382" s="5"/>
       <c r="M382" s="5"/>
@@ -9197,15 +9269,15 @@
     </row>
     <row r="383" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B383" s="10"/>
       <c r="C383" s="10"/>
       <c r="D383" s="19" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E383" s="19" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F383" s="10"/>
       <c r="G383" s="10"/>
@@ -9239,7 +9311,7 @@
     </row>
     <row r="385" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A385" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="2"/>
@@ -9257,7 +9329,7 @@
     </row>
     <row r="386" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A386" s="6" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -9273,72 +9345,72 @@
   <sheetData>
     <row r="8" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E8" s="25" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E15" s="25" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E19" s="25" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E23" s="25" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -9357,23 +9429,23 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F2" s="31" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
@@ -9381,18 +9453,18 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C5" s="25" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -9412,7 +9484,7 @@
         <v>2020</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I7">
         <v>2016</v>
@@ -9430,7 +9502,7 @@
         <v>2020</v>
       </c>
       <c r="N7" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="O7">
         <v>2016</v>
@@ -9448,15 +9520,15 @@
         <v>2020</v>
       </c>
       <c r="T7" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C8" s="34">
         <v>142352</v>
@@ -9523,10 +9595,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B9" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C9" s="33">
         <v>11521</v>
@@ -9593,10 +9665,10 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C10" s="33">
         <v>77862</v>
@@ -9663,10 +9735,10 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B11" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C11" s="33">
         <v>2564</v>
@@ -9733,10 +9805,10 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B12" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C12" s="33">
         <v>32168</v>
@@ -9803,18 +9875,18 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C14" s="25" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
@@ -9834,7 +9906,7 @@
         <v>2020</v>
       </c>
       <c r="H16" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I16">
         <v>2016</v>
@@ -9852,7 +9924,7 @@
         <v>2020</v>
       </c>
       <c r="N16" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="O16">
         <v>2016</v>
@@ -9870,15 +9942,15 @@
         <v>2020</v>
       </c>
       <c r="T16" s="32" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B17" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C17" s="33">
         <v>9962</v>
@@ -9950,4 +10022,24 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>